<commit_message>
Fix: corregir XML para que Excel abra sin advertencia de reparación
</commit_message>
<xml_diff>
--- a/Excel_Automatizado_RM_PRO.xlsx
+++ b/Excel_Automatizado_RM_PRO.xlsx
@@ -1294,7 +1294,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:ns0="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -2073,7 +2073,7 @@
       </c>
     </row>
   </sheetData>
-  <drawing ns0:id="rId1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix: eliminar dibujos PNG que causaban error de reparación en Excel
</commit_message>
<xml_diff>
--- a/Excel_Automatizado_RM_PRO.xlsx
+++ b/Excel_Automatizado_RM_PRO.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="301">
   <si>
     <t xml:space="preserve">PROPIEDADES DE SECCIÓN TRANSVERSAL</t>
   </si>
@@ -47,6 +47,12 @@
     <t xml:space="preserve">Radio de la sección circular. Dato principal de entrada.</t>
   </si>
   <si>
+    <t xml:space="preserve">    ●</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  (   )</t>
+  </si>
+  <si>
     <t xml:space="preserve">   RESULTADOS AUTOMÁTICOS:</t>
   </si>
   <si>
@@ -98,12 +104,18 @@
     <t xml:space="preserve">Radio externo del tubo. Define el tamaño total.</t>
   </si>
   <si>
+    <t xml:space="preserve">  ◎</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Paso 2: Radio interior (r)</t>
   </si>
   <si>
     <t xml:space="preserve">Radio interno (hueco). El espesor = R - r.</t>
   </si>
   <si>
+    <t xml:space="preserve"> (○)</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Paso 3: Área (A = π(R²-r²))</t>
   </si>
   <si>
@@ -137,6 +149,12 @@
     <t xml:space="preserve">Longitud del lado del cuadrado.</t>
   </si>
   <si>
+    <t xml:space="preserve">  ■</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> [  ]</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Paso 2: Área (A = a²)</t>
   </si>
   <si>
@@ -170,12 +188,18 @@
     <t xml:space="preserve">Dimensión exterior del perfil tubular cuadrado.</t>
   </si>
   <si>
+    <t xml:space="preserve">  ▣</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Paso 2: Lado interior (a_int)</t>
   </si>
   <si>
     <t xml:space="preserve">Dimensión interior. Espesor de pared = (a_ext - a_int)/2.</t>
   </si>
   <si>
+    <t xml:space="preserve"> [□]</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Paso 3: Área (A = a_ext² - a_int²)</t>
   </si>
   <si>
@@ -206,12 +230,18 @@
     <t xml:space="preserve">Ancho de la sección (dimensión horizontal).</t>
   </si>
   <si>
+    <t xml:space="preserve">  ▬</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Paso 2: Altura (h)</t>
   </si>
   <si>
     <t xml:space="preserve">Alto de la sección (dimensión vertical).</t>
   </si>
   <si>
+    <t xml:space="preserve"> [==]</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Paso 3: Área (A = b·h)</t>
   </si>
   <si>
@@ -263,10 +293,16 @@
     <t xml:space="preserve">Ancho exterior del perfil.</t>
   </si>
   <si>
+    <t xml:space="preserve">  ▭</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Paso 2: Altura exterior (h_ext)</t>
   </si>
   <si>
     <t xml:space="preserve">Altura exterior del perfil.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> [═]</t>
   </si>
   <si>
     <t xml:space="preserve">   Paso 3: Base interior (b_int)</t>
@@ -1096,203 +1132,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Img1"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Img2"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Img3"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Img4"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>54</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Img5"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>50000</xdr:colOff>
-      <xdr:row>68</xdr:row>
-      <xdr:rowOff>50000</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Img6"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
@@ -1355,10 +1194,18 @@
       <c r="D8" s="9" t="s">
         <v>10</v>
       </c>
+      <c r="E8" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="E9" s="8" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1366,7 +1213,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B11" s="6">
         <f>2*B8</f>
@@ -1375,54 +1222,54 @@
         <v>9</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B12" s="6">
         <f>PI()*B8^2</f>
       </c>
       <c r="C12" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B13" s="6">
         <f>PI()*B8^4/4</f>
       </c>
       <c r="C13" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B14" s="6">
         <f>PI()*B8^3/4</f>
       </c>
       <c r="C14" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15" s="6">
         <f>B8/2</f>
@@ -1431,12 +1278,12 @@
         <v>9</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -1452,7 +1299,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B19" s="4">
         <v>0.075</v>
@@ -1461,12 +1308,15 @@
         <v>9</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B20" s="4">
         <v>0.065</v>
@@ -1475,12 +1325,15 @@
         <v>9</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1488,49 +1341,49 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B23" s="6">
         <f>PI()*(B19^2-B20^2)</f>
       </c>
       <c r="C23" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B24" s="6">
         <f>PI()*(B19^4-B20^4)/4</f>
       </c>
       <c r="C24" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B25" s="6">
         <f>(PI()*(B19^4-B20^4)/4)/B19</f>
       </c>
       <c r="C25" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B26" s="6">
         <f>SQRT((PI()*(B19^4-B20^4)/4)/(PI()*(B19^2-B20^2)))</f>
@@ -1539,12 +1392,12 @@
         <v>9</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1560,7 +1413,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B30" s="4">
         <v>0.1</v>
@@ -1569,12 +1422,20 @@
         <v>9</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>40</v>
+        <v>44</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31" s="8" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -1582,49 +1443,49 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B33" s="6">
         <f>B30^2</f>
       </c>
       <c r="C33" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B34" s="6">
         <f>B30^4/12</f>
       </c>
       <c r="C34" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B35" s="6">
         <f>B30^3/6</f>
       </c>
       <c r="C35" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B36" s="6">
         <f>B30/SQRT(12)</f>
@@ -1633,12 +1494,12 @@
         <v>9</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -1654,7 +1515,7 @@
     </row>
     <row r="40">
       <c r="A40" s="3" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B40" s="4">
         <v>0.12</v>
@@ -1663,12 +1524,15 @@
         <v>9</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>51</v>
+        <v>57</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B41" s="4">
         <v>0.1</v>
@@ -1677,12 +1541,15 @@
         <v>9</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>53</v>
+        <v>60</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
@@ -1690,49 +1557,49 @@
     </row>
     <row r="44">
       <c r="A44" s="3" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B44" s="6">
         <f>B40^2-B41^2</f>
       </c>
       <c r="C44" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="B45" s="6">
         <f>(B40^4-B41^4)/12</f>
       </c>
       <c r="C45" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B46" s="6">
         <f>((B40^4-B41^4)/12)/(B40/2)</f>
       </c>
       <c r="C46" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B47" s="6">
         <f>SQRT(((B40^4-B41^4)/12)/(B40^2-B41^2))</f>
@@ -1741,12 +1608,12 @@
         <v>9</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -1762,7 +1629,7 @@
     </row>
     <row r="51">
       <c r="A51" s="3" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B51" s="4">
         <v>0.08</v>
@@ -1771,12 +1638,15 @@
         <v>9</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>63</v>
+        <v>71</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="B52" s="4">
         <v>0.15</v>
@@ -1785,12 +1655,15 @@
         <v>9</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>65</v>
+        <v>74</v>
+      </c>
+      <c r="E52" s="8" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
@@ -1798,77 +1671,77 @@
     </row>
     <row r="55">
       <c r="A55" s="3" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="B55" s="6">
         <f>B51*B52</f>
       </c>
       <c r="C55" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="B56" s="6">
         <f>B51*B52^3/12</f>
       </c>
       <c r="C56" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="B57" s="6">
         <f>B52*B51^3/12</f>
       </c>
       <c r="C57" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="B58" s="6">
         <f>B51*B52^2/6</f>
       </c>
       <c r="C58" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B59" s="6">
         <f>B52*B51^2/6</f>
       </c>
       <c r="C59" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B60" s="6">
         <f>B52/SQRT(12)</f>
@@ -1877,12 +1750,12 @@
         <v>9</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="B61" s="6">
         <f>B51/SQRT(12)</f>
@@ -1891,12 +1764,12 @@
         <v>9</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -1912,7 +1785,7 @@
     </row>
     <row r="65">
       <c r="A65" s="3" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="B65" s="4">
         <v>0.12</v>
@@ -1921,12 +1794,15 @@
         <v>9</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>82</v>
+        <v>92</v>
+      </c>
+      <c r="E65" s="8" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="B66" s="4">
         <v>0.2</v>
@@ -1935,12 +1811,15 @@
         <v>9</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>84</v>
+        <v>95</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="B67" s="4">
         <v>0.1</v>
@@ -1949,12 +1828,12 @@
         <v>9</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="B68" s="4">
         <v>0.18</v>
@@ -1963,12 +1842,12 @@
         <v>9</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B70" s="5"/>
       <c r="C70" s="5"/>
@@ -1976,77 +1855,77 @@
     </row>
     <row r="71">
       <c r="A71" s="3" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="B71" s="6">
         <f>B65*B66-B67*B68</f>
       </c>
       <c r="C71" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B72" s="6">
         <f>(B65*B66^3-B67*B68^3)/12</f>
       </c>
       <c r="C72" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B73" s="6">
         <f>(B66*B65^3-B68*B67^3)/12</f>
       </c>
       <c r="C73" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="B74" s="6">
         <f>((B65*B66^3-B67*B68^3)/12)/(B66/2)</f>
       </c>
       <c r="C74" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="B75" s="6">
         <f>((B66*B65^3-B68*B67^3)/12)/(B65/2)</f>
       </c>
       <c r="C75" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="B76" s="6">
         <f>SQRT(((B65*B66^3-B67*B68^3)/12)/(B65*B66-B67*B68))</f>
@@ -2055,12 +1934,12 @@
         <v>9</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="B77" s="6">
         <f>SQRT(((B66*B65^3-B68*B67^3)/12)/(B65*B66-B67*B68))</f>
@@ -2069,11 +1948,10 @@
         <v>9</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2088,7 +1966,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2">
@@ -2098,92 +1976,92 @@
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="B6" s="4">
         <v>200</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="B7" s="4">
         <v>345</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="B8" s="4">
         <v>0.0074</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="B9" s="4">
         <v>8.73e-05</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="B10" s="4">
         <v>1.88e-05</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="B11" s="4">
         <v>12.0</v>
@@ -2192,26 +2070,26 @@
         <v>9</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="B12" s="4">
         <v>1.0</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="B13" s="4">
         <v>12.0</v>
@@ -2220,26 +2098,26 @@
         <v>9</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="B14" s="4">
         <v>1.0</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="B15" s="4">
         <v>6.0</v>
@@ -2248,64 +2126,64 @@
         <v>9</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="B16" s="4">
         <v>2.0</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="B19" s="6">
         <f>B6*1E9</f>
       </c>
       <c r="C19" s="10" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="B20" s="6">
         <f>B7*1E6</f>
       </c>
       <c r="C20" s="10" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="B21" s="6">
         <f>B11*B12</f>
@@ -2314,12 +2192,12 @@
         <v>9</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="B22" s="6">
         <f>B13*B14</f>
@@ -2328,144 +2206,144 @@
         <v>9</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="B23" s="6">
         <f>PI()^2*B19*B9/(B21^2)</f>
       </c>
       <c r="C23" s="10" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="B24" s="6">
         <f>PI()^2*B19*B10/(B22^2)</f>
       </c>
       <c r="C24" s="10" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="B25" s="6">
         <f>IF(B23&lt;B24,"Eje x (fuerte)","Eje y (débil)")</f>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="9" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B26" s="6">
         <f>MIN(B23,B24)</f>
       </c>
       <c r="C26" s="10" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B29" s="6">
         <f>B26/B8</f>
       </c>
       <c r="C29" s="10" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="B30" s="6">
         <f>B29/1E6</f>
       </c>
       <c r="C30" s="10" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="B31" s="6">
         <f>B20*B8</f>
       </c>
       <c r="C31" s="10" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="B32" s="6">
         <f>IF(B30&lt;B7,"SI — Rige pandeo (Euler)","NO — Rige fluencia")</f>
       </c>
       <c r="C32" s="10"/>
       <c r="D32" s="9" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="B33" s="6">
         <f>IF(B30&lt;B7,B26,B31)</f>
       </c>
       <c r="C33" s="10" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -2473,44 +2351,44 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B36" s="6">
         <f>B33/B15</f>
       </c>
       <c r="C36" s="10" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="B37" s="6">
         <f>B36/1000</f>
       </c>
       <c r="C37" s="10" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="B39" s="13">
         <f>B37</f>
       </c>
       <c r="C39" s="6" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -2546,85 +2424,85 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="K4" s="11" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="L4" s="11" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="O4" s="11" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="P4" s="11" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="Q4" s="11" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="R4" s="11" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="S4" s="11" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="T4" s="11" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="U4" s="11" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="V4" s="11" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5">
@@ -2632,7 +2510,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="C5" s="4">
         <v>200</v>
@@ -3129,17 +3007,17 @@
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -3159,86 +3037,86 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="14" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="B6" s="4">
         <v>200</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="D6" s="6">
         <f>B6*1E9</f>
       </c>
       <c r="E6" s="10" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="B7" s="4">
         <v>250</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="D7" s="6">
         <f>B7*1E6</f>
       </c>
       <c r="E7" s="10" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="B8" s="4">
         <v>2</v>
       </c>
       <c r="C8" s="10"/>
       <c r="F8" s="9" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -3246,7 +3124,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="B11" s="4">
         <v>2</v>
@@ -3257,7 +3135,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="B12" s="4">
         <v>2.5</v>
@@ -3268,7 +3146,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="B13" s="4">
         <v>3.5</v>
@@ -3279,7 +3157,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -3287,13 +3165,13 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="B16" s="4">
         <v>13</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="D16" s="6">
         <f>B16/100</f>
@@ -3304,13 +3182,13 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="B17" s="4">
         <v>15</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="D17" s="6">
         <f>B17/100</f>
@@ -3321,45 +3199,45 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="F19" s="2" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="B20" s="6">
         <f>PI()*(D17^4-D16^4)/64</f>
       </c>
       <c r="C20" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="B21" s="6">
         <f>PI()*(D17^2-D16^2)/4</f>
       </c>
       <c r="C21" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="B22" s="6">
         <f>SQRT(B20/B21)</f>
@@ -3368,38 +3246,38 @@
         <v>9</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="B23" s="6">
         <f>SQRT(2*PI()^2*D6/D7)</f>
       </c>
       <c r="C23" s="10"/>
       <c r="F23" s="9" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="B26" s="6">
         <f>B8*B11</f>
@@ -3419,7 +3297,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B27" s="6">
         <f>B26/B22</f>
@@ -3434,13 +3312,13 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="B28" s="6">
         <f>PI()^2*D6*B20/B26^2</f>
       </c>
       <c r="C28" s="10" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="D28" s="6">
         <f>PI()^2*D6*B20/D26^2</f>
@@ -3451,13 +3329,13 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="B29" s="13">
         <f>B28/1000</f>
       </c>
       <c r="C29" s="10" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="D29" s="13">
         <f>D28/1000</f>
@@ -3468,13 +3346,13 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="B30" s="6">
         <f>B28/B21/1E6</f>
       </c>
       <c r="C30" s="10" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="D30" s="6">
         <f>D28/B21/1E6</f>
@@ -3485,23 +3363,23 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" s="2" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="B33" s="6">
         <f>B27</f>
@@ -3515,7 +3393,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="B34" s="6">
         <f>IF(B33&lt;B23,"Corta","Larga")</f>
@@ -3529,7 +3407,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="B36" s="6">
         <f>IF(B33&lt;B23,(D7*(1-B33^2/(2*B23^2)))/(5/3+3*B33/(8*B23)-B33^3/(8*B23^3)),(12*PI()^2*D6/(23*B33^2)))/1E6</f>
@@ -3543,7 +3421,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="B37" s="13">
         <f>B36*1E6*B21/1000</f>
@@ -3570,114 +3448,114 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="14" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="B6" s="4">
         <v>30000000</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="B7" s="4">
         <v>20000</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="B10" s="4">
         <v>1</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B11" s="4">
         <v>0.7</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="B12" s="4">
         <v>0.5</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="B13" s="4">
         <v>2</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -3685,7 +3563,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="B16" s="4">
         <v>2.5</v>
@@ -3694,68 +3572,68 @@
         <v>9</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="B17" s="6">
         <f>B16*39.3701</f>
       </c>
       <c r="C17" s="10" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="B18" s="4">
         <v>17.6</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="B19" s="4">
         <v>116</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="B20" s="4">
         <v>2.57</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -3763,39 +3641,39 @@
     </row>
     <row r="23">
       <c r="A23" s="11" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="B24" s="6">
         <f>B10</f>
@@ -3827,7 +3705,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="B25" s="6">
         <f>B11</f>
@@ -3859,7 +3737,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="B26" s="6">
         <f>B12</f>
@@ -3891,7 +3769,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="B27" s="6">
         <f>B13</f>

</xml_diff>